<commit_message>
Added 1 Group Events
</commit_message>
<xml_diff>
--- a/input files/player_list.xlsx
+++ b/input files/player_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tkdma\Documents\Projects\Ranking_and_Draw\input files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding\Programming Projects\Python\Ranking_and_Draw\input files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE14073F-6BD6-4849-9C15-62F4E2936CC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B42FF761-18C2-41CE-BDC3-B63C350882CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="u11b" sheetId="2" r:id="rId1"/>
@@ -21,11 +21,12 @@
     <sheet name="cadet girls" sheetId="7" r:id="rId6"/>
     <sheet name="jnr boys" sheetId="8" r:id="rId7"/>
     <sheet name="jnr girls" sheetId="9" r:id="rId8"/>
-    <sheet name="u21m" sheetId="10" r:id="rId9"/>
-    <sheet name="u21w" sheetId="11" r:id="rId10"/>
-    <sheet name="mens singles" sheetId="1" r:id="rId11"/>
-    <sheet name="womens singles" sheetId="12" r:id="rId12"/>
-    <sheet name="senior mxs" sheetId="13" r:id="rId13"/>
+    <sheet name="jnr mxs" sheetId="14" r:id="rId9"/>
+    <sheet name="u21m" sheetId="10" r:id="rId10"/>
+    <sheet name="u21w" sheetId="11" r:id="rId11"/>
+    <sheet name="mens singles" sheetId="1" r:id="rId12"/>
+    <sheet name="womens singles" sheetId="12" r:id="rId13"/>
+    <sheet name="senior mxs" sheetId="13" r:id="rId14"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="43">
   <si>
     <t>Licence Number</t>
   </si>
@@ -46,19 +47,145 @@
   </si>
   <si>
     <t>County</t>
+  </si>
+  <si>
+    <t>Abu Sami Mohammad Osman</t>
+  </si>
+  <si>
+    <t>Dexter Barber</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>Louis Green</t>
+  </si>
+  <si>
+    <t>Shalen Auckloo</t>
+  </si>
+  <si>
+    <t>Dhruv Datta</t>
+  </si>
+  <si>
+    <t>Sy</t>
+  </si>
+  <si>
+    <t>Ca</t>
+  </si>
+  <si>
+    <t>Mx</t>
+  </si>
+  <si>
+    <t>Bd</t>
+  </si>
+  <si>
+    <t>Do</t>
+  </si>
+  <si>
+    <t>Ys</t>
+  </si>
+  <si>
+    <t>Bk</t>
+  </si>
+  <si>
+    <t>Charlton Ngitngit</t>
+  </si>
+  <si>
+    <t>Lewis Salmon</t>
+  </si>
+  <si>
+    <t>Euan Hacking</t>
+  </si>
+  <si>
+    <t>Aarav Singh</t>
+  </si>
+  <si>
+    <t>Edward Hatton</t>
+  </si>
+  <si>
+    <t>Noah Byrne-Smith</t>
+  </si>
+  <si>
+    <t>James Roberts</t>
+  </si>
+  <si>
+    <t>Sebastian Runcanu</t>
+  </si>
+  <si>
+    <t>Connor Shearing</t>
+  </si>
+  <si>
+    <t>Ethan Ang</t>
+  </si>
+  <si>
+    <t>Vihan Nirmal</t>
+  </si>
+  <si>
+    <t>Ishaan Sethi</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>Vardhini Nishanth</t>
+  </si>
+  <si>
+    <t>Lydia White</t>
+  </si>
+  <si>
+    <t>Evie Knaapen</t>
+  </si>
+  <si>
+    <t>Wa</t>
+  </si>
+  <si>
+    <t>Li</t>
+  </si>
+  <si>
+    <t>Zhaoen Sean Wang</t>
+  </si>
+  <si>
+    <t>Louis Alexander</t>
+  </si>
+  <si>
+    <t>Omar Faruqe Wasi</t>
+  </si>
+  <si>
+    <t>Troy Williams</t>
+  </si>
+  <si>
+    <t>Joshua Fernandes</t>
+  </si>
+  <si>
+    <t>Ben Levi</t>
+  </si>
+  <si>
+    <t>Wadjid Wafiq</t>
+  </si>
+  <si>
+    <t>Gregory Fray</t>
+  </si>
+  <si>
+    <t>Jaydan Griffiths</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -81,12 +208,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -368,9 +504,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7195429-0F42-4326-B440-D9F66DA5018B}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -387,11 +523,11 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B86FE96B-5CB4-470F-9324-E97AC5632FFA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F99962-8D69-4C57-A6B0-D7EC5BAE272F}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -408,14 +544,11 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="33.44140625" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B86FE96B-5CB4-470F-9324-E97AC5632FFA}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -425,12 +558,6 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C3" s="2"/>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B21" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -438,11 +565,15 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C28D3487-43C4-4AA0-8786-3EE79B33E419}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="33.453125" customWidth="1"/>
+    <col min="3" max="3" width="19.26953125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -459,15 +590,11 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{174C7096-5BC0-4B77-8308-7CEB2388EFCE}">
-  <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="24.44140625" customWidth="1"/>
-    <col min="3" max="3" width="20.33203125" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C28D3487-43C4-4AA0-8786-3EE79B33E419}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -477,24 +604,43 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C3" s="2"/>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B21" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{174C7096-5BC0-4B77-8308-7CEB2388EFCE}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="24.453125" customWidth="1"/>
+    <col min="3" max="3" width="20.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7C0B9A5-B02C-4FE9-AB7E-590CD0BB78A9}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -513,9 +659,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{718486FE-0BE7-45E6-96E5-39901D3E2F43}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -534,9 +680,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35B1F53A-9442-44FA-87EA-BBD2789806E7}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -554,10 +700,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDCF8AB2-0D09-4A4D-9990-281AC0707992}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="16.08984375" customWidth="1"/>
+    <col min="2" max="2" width="37" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -566,6 +716,193 @@
       </c>
       <c r="C1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="3">
+        <v>315881</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="3">
+        <v>999999999</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="3">
+        <v>315678</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="3">
+        <v>315680</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="3">
+        <v>311394</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="3">
+        <v>306559</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="3">
+        <v>317767</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="3">
+        <v>302423</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="3">
+        <v>308761</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="3">
+        <v>310263</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="3">
+        <v>306924</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="3">
+        <v>313884</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="3">
+        <v>313281</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="3">
+        <v>317728</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="3">
+        <v>999999999</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="3">
+        <v>314533</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" s="3">
+        <v>317252</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -575,10 +912,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E10BE8C-58FA-45C1-9940-1F0EBE34B3CB}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="16.08984375" customWidth="1"/>
+    <col min="2" max="2" width="21.08984375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -587,6 +928,39 @@
       </c>
       <c r="C1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>300391</v>
+      </c>
+      <c r="B2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>187238</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>9999999999</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -596,10 +970,14 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1069734F-3B45-457C-8E0F-1E6A65F3E6B6}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="24.36328125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -609,6 +987,66 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="5"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="4"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="4"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="4"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="4"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="4"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="4"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="4"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="4"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="4"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="4"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="4"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="4"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="4"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="4"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="4"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="4"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="4"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="4"/>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -618,9 +1056,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1A94DB7-3AB9-4026-B094-75E91B1DD63C}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.1796875" customWidth="1"/>
+    <col min="2" max="2" width="8.7265625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -637,11 +1079,15 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F99962-8D69-4C57-A6B0-D7EC5BAE272F}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80D042EA-0286-46F2-AF2D-9079E1EFF0A5}">
+  <dimension ref="A1:C22"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.90625" customWidth="1"/>
+    <col min="2" max="2" width="36" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -650,6 +1096,237 @@
       </c>
       <c r="C1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="5">
+        <v>310833</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="4">
+        <v>303200</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>315880</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>315881</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>188115</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
+        <v>306559</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>317767</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>308761</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
+        <v>310263</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
+        <v>306924</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>313884</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
+        <v>203194</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="4">
+        <v>197542</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
+        <v>184606</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="4">
+        <v>192131</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
+        <v>311773</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>9999999999</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="4">
+        <v>313281</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="4">
+        <v>314533</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>300391</v>
+      </c>
+      <c r="B21" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>9999999999</v>
+      </c>
+      <c r="B22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>